<commit_message>
nueva asignacion y cantidad lhd
</commit_message>
<xml_diff>
--- a/data/Escenarios_DET/carga_on_board_costo_fijo/elmo_data.xlsx
+++ b/data/Escenarios_DET/carga_on_board_costo_fijo/elmo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agustin\Desktop\Elmo_infrastructure_NP\data\DET\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Escenarios_DET\carga_on_board_costo_fijo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4BF981E-4743-4260-8081-0B198CFC98F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF88FB80-B49F-46D6-A102-2AF6FDD6CC63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6000" yWindow="4185" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="305">
   <si>
     <t>id</t>
   </si>
@@ -952,12 +952,6 @@
   </si>
   <si>
     <t>LH518B_7</t>
-  </si>
-  <si>
-    <t>LH518B_8</t>
-  </si>
-  <si>
-    <t>LH518B_9</t>
   </si>
 </sst>
 </file>
@@ -1791,39 +1785,39 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AD11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AD9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" style="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.33203125" style="20" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" style="20" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5546875" style="20" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.44140625" style="20" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.77734375" style="62" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5546875" style="20" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" style="21" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.109375" style="20" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" style="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.28515625" style="20" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" style="20" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5703125" style="20" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.42578125" style="20" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.7109375" style="62" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5703125" style="20" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" style="21" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" style="20" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="15" style="20" customWidth="1"/>
-    <col min="16" max="16" width="16.88671875" style="20" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.77734375" style="21" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.85546875" style="20" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.7109375" style="21" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="18" style="21" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="20.88671875" style="21" bestFit="1" customWidth="1"/>
-    <col min="20" max="23" width="20.88671875" style="21" customWidth="1"/>
-    <col min="24" max="24" width="18.44140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="20.109375" style="21" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.21875" style="21" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8.21875" style="21" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="20" max="23" width="20.85546875" style="21" customWidth="1"/>
+    <col min="24" max="24" width="18.42578125" style="21" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="20.140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.28515625" style="21" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.28515625" style="21" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1915,7 +1909,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
         <v>3</v>
       </c>
@@ -2007,7 +2001,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:30" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="28">
         <v>1</v>
       </c>
@@ -2099,7 +2093,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="28">
         <v>2</v>
       </c>
@@ -2191,7 +2185,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="28">
         <v>3</v>
       </c>
@@ -2283,7 +2277,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="28">
         <v>4</v>
       </c>
@@ -2375,7 +2369,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="28">
         <v>5</v>
       </c>
@@ -2467,7 +2461,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="28">
         <v>6</v>
       </c>
@@ -2559,7 +2553,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="28">
         <v>7</v>
       </c>
@@ -2648,190 +2642,6 @@
         <v>0.95</v>
       </c>
       <c r="AD9" s="65">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A10" s="28">
-        <v>8</v>
-      </c>
-      <c r="B10" s="33" t="s">
-        <v>305</v>
-      </c>
-      <c r="C10" s="31" t="s">
-        <v>73</v>
-      </c>
-      <c r="D10" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="G10" s="6">
-        <v>18</v>
-      </c>
-      <c r="H10" s="63">
-        <v>0.84</v>
-      </c>
-      <c r="I10" s="64">
-        <v>20</v>
-      </c>
-      <c r="J10" s="64">
-        <v>20</v>
-      </c>
-      <c r="K10" s="61">
-        <v>54.8</v>
-      </c>
-      <c r="L10" s="6">
-        <v>540</v>
-      </c>
-      <c r="M10" s="19">
-        <v>8.73</v>
-      </c>
-      <c r="N10" s="58">
-        <v>-1</v>
-      </c>
-      <c r="O10" s="58">
-        <v>-1</v>
-      </c>
-      <c r="P10" s="58">
-        <v>-1</v>
-      </c>
-      <c r="Q10" s="58">
-        <v>-1</v>
-      </c>
-      <c r="R10" s="32">
-        <v>0.95</v>
-      </c>
-      <c r="S10" s="23">
-        <v>0.92</v>
-      </c>
-      <c r="T10" s="25">
-        <v>15</v>
-      </c>
-      <c r="U10" s="66">
-        <v>0.47</v>
-      </c>
-      <c r="V10" s="31">
-        <v>160</v>
-      </c>
-      <c r="W10" s="65">
-        <v>4</v>
-      </c>
-      <c r="X10" s="57">
-        <v>320</v>
-      </c>
-      <c r="Y10" s="67">
-        <v>4</v>
-      </c>
-      <c r="Z10" s="57">
-        <v>482</v>
-      </c>
-      <c r="AA10" s="57">
-        <v>0.2</v>
-      </c>
-      <c r="AB10" s="65">
-        <v>0.95</v>
-      </c>
-      <c r="AC10" s="65">
-        <v>0.95</v>
-      </c>
-      <c r="AD10" s="65">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A11" s="28">
-        <v>9</v>
-      </c>
-      <c r="B11" s="33" t="s">
-        <v>306</v>
-      </c>
-      <c r="C11" s="31" t="s">
-        <v>73</v>
-      </c>
-      <c r="D11" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="G11" s="6">
-        <v>18</v>
-      </c>
-      <c r="H11" s="63">
-        <v>0.84</v>
-      </c>
-      <c r="I11" s="64">
-        <v>20</v>
-      </c>
-      <c r="J11" s="64">
-        <v>20</v>
-      </c>
-      <c r="K11" s="61">
-        <v>54.8</v>
-      </c>
-      <c r="L11" s="6">
-        <v>540</v>
-      </c>
-      <c r="M11" s="19">
-        <v>8.73</v>
-      </c>
-      <c r="N11" s="58">
-        <v>-1</v>
-      </c>
-      <c r="O11" s="58">
-        <v>-1</v>
-      </c>
-      <c r="P11" s="58">
-        <v>-1</v>
-      </c>
-      <c r="Q11" s="58">
-        <v>-1</v>
-      </c>
-      <c r="R11" s="32">
-        <v>0.95</v>
-      </c>
-      <c r="S11" s="23">
-        <v>0.92</v>
-      </c>
-      <c r="T11" s="25">
-        <v>15</v>
-      </c>
-      <c r="U11" s="66">
-        <v>0.47</v>
-      </c>
-      <c r="V11" s="31">
-        <v>160</v>
-      </c>
-      <c r="W11" s="65">
-        <v>4</v>
-      </c>
-      <c r="X11" s="57">
-        <v>320</v>
-      </c>
-      <c r="Y11" s="67">
-        <v>4</v>
-      </c>
-      <c r="Z11" s="57">
-        <v>482</v>
-      </c>
-      <c r="AA11" s="57">
-        <v>0.2</v>
-      </c>
-      <c r="AB11" s="65">
-        <v>0.95</v>
-      </c>
-      <c r="AC11" s="65">
-        <v>0.95</v>
-      </c>
-      <c r="AD11" s="65">
         <v>8</v>
       </c>
     </row>
@@ -2845,15 +2655,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC93900-5A86-4519-AB89-460E8AC441EE}">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.88671875" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -2876,7 +2686,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
         <v>3</v>
       </c>
@@ -2899,7 +2709,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="31">
         <v>1</v>
       </c>
@@ -2932,14 +2742,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA5C58D2-31A1-4CA6-99E5-3102447D41CF}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -2959,7 +2769,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
         <v>3</v>
       </c>
@@ -2979,7 +2789,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="31">
         <v>1</v>
       </c>
@@ -3010,17 +2820,17 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H236"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="29.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
@@ -3046,7 +2856,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="45" t="s">
         <v>3</v>
       </c>
@@ -3072,7 +2882,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="52">
         <v>1</v>
       </c>
@@ -3098,7 +2908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="52">
         <v>2</v>
       </c>
@@ -3124,7 +2934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="52">
         <v>3</v>
       </c>
@@ -3150,7 +2960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="52">
         <v>4</v>
       </c>
@@ -3176,7 +2986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="52">
         <v>5</v>
       </c>
@@ -3202,7 +3012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="52">
         <v>6</v>
       </c>
@@ -3228,7 +3038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="52">
         <v>7</v>
       </c>
@@ -3254,7 +3064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="52">
         <v>8</v>
       </c>
@@ -3280,7 +3090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="52">
         <v>9</v>
       </c>
@@ -3306,7 +3116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="52">
         <v>10</v>
       </c>
@@ -3332,7 +3142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="52">
         <v>11</v>
       </c>
@@ -3358,7 +3168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="52">
         <v>12</v>
       </c>
@@ -3384,7 +3194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="52">
         <v>13</v>
       </c>
@@ -3410,7 +3220,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="52">
         <v>14</v>
       </c>
@@ -3436,7 +3246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="52">
         <v>15</v>
       </c>
@@ -3462,7 +3272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="52">
         <v>16</v>
       </c>
@@ -3488,7 +3298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="52">
         <v>17</v>
       </c>
@@ -3514,7 +3324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="52">
         <v>18</v>
       </c>
@@ -3540,7 +3350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="52">
         <v>19</v>
       </c>
@@ -3566,7 +3376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="52">
         <v>20</v>
       </c>
@@ -3592,7 +3402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="52">
         <v>21</v>
       </c>
@@ -3618,7 +3428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="52">
         <v>22</v>
       </c>
@@ -3644,7 +3454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="52">
         <v>23</v>
       </c>
@@ -3670,7 +3480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="52">
         <v>24</v>
       </c>
@@ -3696,7 +3506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="52">
         <v>25</v>
       </c>
@@ -3722,7 +3532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="52">
         <v>26</v>
       </c>
@@ -3748,7 +3558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="52">
         <v>27</v>
       </c>
@@ -3774,7 +3584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="52">
         <v>28</v>
       </c>
@@ -3800,7 +3610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="52">
         <v>29</v>
       </c>
@@ -3826,7 +3636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="52">
         <v>30</v>
       </c>
@@ -3852,7 +3662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="52">
         <v>31</v>
       </c>
@@ -3878,7 +3688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="52">
         <v>32</v>
       </c>
@@ -3904,7 +3714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="52">
         <v>33</v>
       </c>
@@ -3930,7 +3740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="52">
         <v>34</v>
       </c>
@@ -3956,7 +3766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="52">
         <v>35</v>
       </c>
@@ -3982,7 +3792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="52">
         <v>36</v>
       </c>
@@ -4008,7 +3818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="52">
         <v>37</v>
       </c>
@@ -4034,7 +3844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="52">
         <v>38</v>
       </c>
@@ -4060,7 +3870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="52">
         <v>39</v>
       </c>
@@ -4086,7 +3896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="52">
         <v>40</v>
       </c>
@@ -4112,7 +3922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="52">
         <v>41</v>
       </c>
@@ -4138,7 +3948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="52">
         <v>42</v>
       </c>
@@ -4164,7 +3974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="52">
         <v>43</v>
       </c>
@@ -4190,7 +4000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="52">
         <v>44</v>
       </c>
@@ -4216,7 +4026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="52">
         <v>45</v>
       </c>
@@ -4242,7 +4052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="52">
         <v>46</v>
       </c>
@@ -4268,7 +4078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="52">
         <v>47</v>
       </c>
@@ -4294,7 +4104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="52">
         <v>48</v>
       </c>
@@ -4320,7 +4130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="52">
         <v>49</v>
       </c>
@@ -4346,7 +4156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="52">
         <v>50</v>
       </c>
@@ -4372,7 +4182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="52">
         <v>51</v>
       </c>
@@ -4398,7 +4208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="52">
         <v>52</v>
       </c>
@@ -4424,7 +4234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="52">
         <v>53</v>
       </c>
@@ -4450,7 +4260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="52">
         <v>54</v>
       </c>
@@ -4476,7 +4286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="52">
         <v>55</v>
       </c>
@@ -4502,7 +4312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="52">
         <v>56</v>
       </c>
@@ -4528,7 +4338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="52">
         <v>57</v>
       </c>
@@ -4554,7 +4364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="52">
         <v>58</v>
       </c>
@@ -4580,7 +4390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="52">
         <v>59</v>
       </c>
@@ -4606,7 +4416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="52">
         <v>60</v>
       </c>
@@ -4632,7 +4442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="52">
         <v>61</v>
       </c>
@@ -4658,7 +4468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="52">
         <v>62</v>
       </c>
@@ -4684,7 +4494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="52">
         <v>63</v>
       </c>
@@ -4710,7 +4520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="52">
         <v>64</v>
       </c>
@@ -4736,7 +4546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="52">
         <v>65</v>
       </c>
@@ -4762,7 +4572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="52">
         <v>66</v>
       </c>
@@ -4788,7 +4598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="52">
         <v>67</v>
       </c>
@@ -4814,7 +4624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="52">
         <v>68</v>
       </c>
@@ -4840,7 +4650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="52">
         <v>69</v>
       </c>
@@ -4866,7 +4676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="52">
         <v>70</v>
       </c>
@@ -4892,7 +4702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="52">
         <v>71</v>
       </c>
@@ -4918,7 +4728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="52">
         <v>72</v>
       </c>
@@ -4944,7 +4754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="52">
         <v>73</v>
       </c>
@@ -4970,7 +4780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="52">
         <v>74</v>
       </c>
@@ -4996,7 +4806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="52">
         <v>75</v>
       </c>
@@ -5022,7 +4832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="52">
         <v>76</v>
       </c>
@@ -5048,7 +4858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="52">
         <v>77</v>
       </c>
@@ -5074,7 +4884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="52">
         <v>78</v>
       </c>
@@ -5100,7 +4910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="52">
         <v>79</v>
       </c>
@@ -5126,7 +4936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="52">
         <v>80</v>
       </c>
@@ -5152,7 +4962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="52">
         <v>81</v>
       </c>
@@ -5178,7 +4988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="52">
         <v>82</v>
       </c>
@@ -5204,7 +5014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="52">
         <v>83</v>
       </c>
@@ -5230,7 +5040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="52">
         <v>84</v>
       </c>
@@ -5256,7 +5066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="52">
         <v>85</v>
       </c>
@@ -5282,7 +5092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="52">
         <v>86</v>
       </c>
@@ -5308,7 +5118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="52">
         <v>87</v>
       </c>
@@ -5334,7 +5144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" s="52">
         <v>88</v>
       </c>
@@ -5360,7 +5170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" s="52">
         <v>89</v>
       </c>
@@ -5386,7 +5196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" s="52">
         <v>90</v>
       </c>
@@ -5412,7 +5222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" s="52">
         <v>91</v>
       </c>
@@ -5438,7 +5248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" s="52">
         <v>92</v>
       </c>
@@ -5464,7 +5274,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="52">
         <v>93</v>
       </c>
@@ -5490,7 +5300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="52">
         <v>94</v>
       </c>
@@ -5516,7 +5326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="52">
         <v>95</v>
       </c>
@@ -5542,7 +5352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="52">
         <v>96</v>
       </c>
@@ -5568,7 +5378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="52">
         <v>97</v>
       </c>
@@ -5594,7 +5404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" s="52">
         <v>98</v>
       </c>
@@ -5620,7 +5430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="52">
         <v>99</v>
       </c>
@@ -5646,7 +5456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" s="52">
         <v>100</v>
       </c>
@@ -5672,7 +5482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" s="52">
         <v>101</v>
       </c>
@@ -5698,7 +5508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" s="52">
         <v>102</v>
       </c>
@@ -5724,7 +5534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" s="52">
         <v>103</v>
       </c>
@@ -5750,7 +5560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" s="52">
         <v>104</v>
       </c>
@@ -5776,7 +5586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" s="52">
         <v>105</v>
       </c>
@@ -5802,7 +5612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" s="52">
         <v>106</v>
       </c>
@@ -5828,7 +5638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" s="52">
         <v>107</v>
       </c>
@@ -5854,7 +5664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" s="52">
         <v>108</v>
       </c>
@@ -5880,7 +5690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" s="52">
         <v>109</v>
       </c>
@@ -5906,7 +5716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" s="52">
         <v>110</v>
       </c>
@@ -5932,7 +5742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" s="52">
         <v>111</v>
       </c>
@@ -5958,7 +5768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" s="52">
         <v>112</v>
       </c>
@@ -5984,7 +5794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" s="52">
         <v>113</v>
       </c>
@@ -6010,7 +5820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" s="52">
         <v>114</v>
       </c>
@@ -6036,7 +5846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" s="52">
         <v>115</v>
       </c>
@@ -6062,7 +5872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" s="52">
         <v>116</v>
       </c>
@@ -6088,7 +5898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" s="52">
         <v>117</v>
       </c>
@@ -6114,7 +5924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" s="52">
         <v>118</v>
       </c>
@@ -6140,7 +5950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121" s="52">
         <v>119</v>
       </c>
@@ -6166,7 +5976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" s="52">
         <v>120</v>
       </c>
@@ -6192,7 +6002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" s="52">
         <v>121</v>
       </c>
@@ -6218,7 +6028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" s="52">
         <v>122</v>
       </c>
@@ -6244,7 +6054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125" s="52">
         <v>123</v>
       </c>
@@ -6270,7 +6080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" s="52">
         <v>124</v>
       </c>
@@ -6296,7 +6106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" s="52">
         <v>125</v>
       </c>
@@ -6322,7 +6132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128" s="52">
         <v>126</v>
       </c>
@@ -6348,7 +6158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A129" s="52">
         <v>127</v>
       </c>
@@ -6374,7 +6184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130" s="52">
         <v>128</v>
       </c>
@@ -6400,7 +6210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A131" s="52">
         <v>129</v>
       </c>
@@ -6426,7 +6236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A132" s="52">
         <v>130</v>
       </c>
@@ -6452,7 +6262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A133" s="52">
         <v>131</v>
       </c>
@@ -6478,7 +6288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A134" s="52">
         <v>132</v>
       </c>
@@ -6504,7 +6314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A135" s="52">
         <v>133</v>
       </c>
@@ -6530,7 +6340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A136" s="52">
         <v>134</v>
       </c>
@@ -6556,7 +6366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A137" s="52">
         <v>135</v>
       </c>
@@ -6582,7 +6392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A138" s="52">
         <v>136</v>
       </c>
@@ -6608,7 +6418,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A139" s="52">
         <v>137</v>
       </c>
@@ -6634,7 +6444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A140" s="52">
         <v>138</v>
       </c>
@@ -6660,7 +6470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A141" s="52">
         <v>139</v>
       </c>
@@ -6686,7 +6496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A142" s="52">
         <v>140</v>
       </c>
@@ -6712,7 +6522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A143" s="52">
         <v>141</v>
       </c>
@@ -6738,7 +6548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A144" s="52">
         <v>142</v>
       </c>
@@ -6764,7 +6574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A145" s="52">
         <v>143</v>
       </c>
@@ -6790,7 +6600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A146" s="52">
         <v>144</v>
       </c>
@@ -6816,7 +6626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A147" s="52">
         <v>145</v>
       </c>
@@ -6842,7 +6652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A148" s="52">
         <v>146</v>
       </c>
@@ -6868,7 +6678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A149" s="52">
         <v>147</v>
       </c>
@@ -6894,7 +6704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A150" s="52">
         <v>148</v>
       </c>
@@ -6920,7 +6730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A151" s="52">
         <v>149</v>
       </c>
@@ -6946,7 +6756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152" s="52">
         <v>150</v>
       </c>
@@ -6972,7 +6782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153" s="52">
         <v>151</v>
       </c>
@@ -6998,7 +6808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154" s="52">
         <v>152</v>
       </c>
@@ -7024,7 +6834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155" s="52">
         <v>153</v>
       </c>
@@ -7050,7 +6860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156" s="52">
         <v>154</v>
       </c>
@@ -7076,7 +6886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157" s="52">
         <v>155</v>
       </c>
@@ -7102,7 +6912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158" s="52">
         <v>156</v>
       </c>
@@ -7128,7 +6938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159" s="52">
         <v>157</v>
       </c>
@@ -7154,7 +6964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160" s="52">
         <v>158</v>
       </c>
@@ -7180,7 +6990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A161" s="52">
         <v>159</v>
       </c>
@@ -7206,7 +7016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A162" s="52">
         <v>160</v>
       </c>
@@ -7232,7 +7042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A163" s="52">
         <v>161</v>
       </c>
@@ -7258,7 +7068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164" s="52">
         <v>162</v>
       </c>
@@ -7284,7 +7094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A165" s="52">
         <v>163</v>
       </c>
@@ -7310,7 +7120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A166" s="52">
         <v>164</v>
       </c>
@@ -7336,7 +7146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A167" s="52">
         <v>165</v>
       </c>
@@ -7362,7 +7172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A168" s="52">
         <v>166</v>
       </c>
@@ -7388,7 +7198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A169" s="52">
         <v>167</v>
       </c>
@@ -7414,7 +7224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A170" s="52">
         <v>168</v>
       </c>
@@ -7440,7 +7250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A171" s="52">
         <v>169</v>
       </c>
@@ -7466,7 +7276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A172" s="52">
         <v>170</v>
       </c>
@@ -7492,7 +7302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A173" s="52">
         <v>171</v>
       </c>
@@ -7518,7 +7328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A174" s="52">
         <v>172</v>
       </c>
@@ -7544,7 +7354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A175" s="52">
         <v>173</v>
       </c>
@@ -7570,7 +7380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A176" s="52">
         <v>174</v>
       </c>
@@ -7596,7 +7406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A177" s="52">
         <v>175</v>
       </c>
@@ -7622,7 +7432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A178" s="52">
         <v>176</v>
       </c>
@@ -7648,7 +7458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A179" s="52">
         <v>177</v>
       </c>
@@ -7674,7 +7484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A180" s="52">
         <v>178</v>
       </c>
@@ -7700,7 +7510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A181" s="52">
         <v>179</v>
       </c>
@@ -7726,7 +7536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A182" s="52">
         <v>180</v>
       </c>
@@ -7752,7 +7562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A183" s="52">
         <v>181</v>
       </c>
@@ -7778,7 +7588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A184" s="52">
         <v>182</v>
       </c>
@@ -7804,7 +7614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A185" s="52">
         <v>183</v>
       </c>
@@ -7830,7 +7640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A186" s="52">
         <v>184</v>
       </c>
@@ -7856,7 +7666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A187" s="52">
         <v>185</v>
       </c>
@@ -7882,7 +7692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A188" s="52">
         <v>186</v>
       </c>
@@ -7908,7 +7718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A189" s="52">
         <v>187</v>
       </c>
@@ -7934,7 +7744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A190" s="52">
         <v>188</v>
       </c>
@@ -7960,7 +7770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A191" s="52">
         <v>189</v>
       </c>
@@ -7986,7 +7796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A192" s="52">
         <v>190</v>
       </c>
@@ -8012,7 +7822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A193" s="52">
         <v>191</v>
       </c>
@@ -8038,7 +7848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A194" s="52">
         <v>192</v>
       </c>
@@ -8064,7 +7874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A195" s="52">
         <v>193</v>
       </c>
@@ -8090,7 +7900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A196" s="52">
         <v>194</v>
       </c>
@@ -8116,7 +7926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A197" s="52">
         <v>195</v>
       </c>
@@ -8142,7 +7952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A198" s="52">
         <v>196</v>
       </c>
@@ -8168,7 +7978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A199" s="52">
         <v>197</v>
       </c>
@@ -8194,7 +8004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A200" s="52">
         <v>198</v>
       </c>
@@ -8220,7 +8030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A201" s="52">
         <v>199</v>
       </c>
@@ -8246,7 +8056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A202" s="52">
         <v>200</v>
       </c>
@@ -8272,7 +8082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A203" s="52">
         <v>201</v>
       </c>
@@ -8298,7 +8108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A204" s="52">
         <v>202</v>
       </c>
@@ -8324,7 +8134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A205" s="52">
         <v>203</v>
       </c>
@@ -8350,7 +8160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A206" s="52">
         <v>204</v>
       </c>
@@ -8376,7 +8186,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A207" s="52">
         <v>205</v>
       </c>
@@ -8402,7 +8212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A208" s="52">
         <v>206</v>
       </c>
@@ -8428,7 +8238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A209" s="52">
         <v>207</v>
       </c>
@@ -8454,7 +8264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A210" s="52">
         <v>208</v>
       </c>
@@ -8480,7 +8290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A211" s="52">
         <v>209</v>
       </c>
@@ -8506,7 +8316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A212" s="52">
         <v>210</v>
       </c>
@@ -8532,90 +8342,90 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A213"/>
       <c r="C213"/>
       <c r="D213"/>
       <c r="G213"/>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A214"/>
       <c r="C214"/>
       <c r="D214"/>
       <c r="G214"/>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A215"/>
       <c r="C215"/>
       <c r="D215"/>
       <c r="G215"/>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A216"/>
       <c r="C216"/>
       <c r="D216"/>
       <c r="G216"/>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A217"/>
       <c r="C217"/>
       <c r="D217"/>
       <c r="G217"/>
     </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A218"/>
       <c r="C218"/>
       <c r="D218"/>
       <c r="G218"/>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A219"/>
       <c r="C219"/>
       <c r="D219"/>
       <c r="G219"/>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A220"/>
       <c r="C220"/>
       <c r="D220"/>
       <c r="G220"/>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A221"/>
       <c r="C221"/>
       <c r="D221"/>
       <c r="G221"/>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A222"/>
       <c r="C222"/>
       <c r="D222"/>
       <c r="G222"/>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A223"/>
       <c r="C223"/>
       <c r="D223"/>
       <c r="G223"/>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A224"/>
       <c r="C224"/>
       <c r="D224"/>
       <c r="G224"/>
     </row>
-    <row r="225" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="226" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="227" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="228" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="229" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="230" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="231" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="232" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="233" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="234" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="235" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="236" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="225" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="226" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="227" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="228" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="229" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="230" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="231" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="232" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="233" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="234" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="235" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="236" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8628,14 +8438,14 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8646,7 +8456,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -8657,7 +8467,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>0</v>
       </c>

</xml_diff>